<commit_message>
Auto update Pengadaan 2026-09-01 08:10:02
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-01).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-01).xlsx
@@ -10201,7 +10201,7 @@
         <v>1559826000</v>
       </c>
       <c r="I65" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J65" s="6" t="n">
         <v>1559826000</v>
@@ -10299,7 +10299,7 @@
         <v>64526744076.01</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J67" s="13" t="n">
         <v>60467810276</v>

</xml_diff>